<commit_message>
app totalmente funcional CRUD, login,logout,autenticacion con token jwt,rutas proteginas con jwt
</commit_message>
<xml_diff>
--- a/frontend/public/plantillaFormato.xlsx
+++ b/frontend/public/plantillaFormato.xlsx
@@ -476,12 +476,70 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -491,15 +549,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -518,60 +567,26 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1445,8 +1460,8 @@
     <col min="8" max="25" width="10.90625" style="13"/>
     <col min="26" max="26" width="17.6328125" style="13" customWidth="1"/>
     <col min="27" max="27" width="25.90625" style="13" customWidth="1"/>
-    <col min="28" max="28" width="18.36328125" style="45" customWidth="1"/>
-    <col min="29" max="29" width="21.453125" style="45" customWidth="1"/>
+    <col min="28" max="28" width="18.36328125" style="19" customWidth="1"/>
+    <col min="29" max="29" width="21.453125" style="19" customWidth="1"/>
     <col min="30" max="30" width="19.1796875" style="13" customWidth="1"/>
     <col min="31" max="31" width="17.54296875" style="13" customWidth="1"/>
     <col min="32" max="32" width="20.453125" style="13" customWidth="1"/>
@@ -1461,7 +1476,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:42" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="17"/>
+      <c r="A1" s="37"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="2"/>
@@ -1488,8 +1503,8 @@
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
       <c r="AA1" s="2"/>
-      <c r="AB1" s="41"/>
-      <c r="AC1" s="41"/>
+      <c r="AB1" s="17"/>
+      <c r="AC1" s="17"/>
       <c r="AD1" s="2"/>
       <c r="AE1" s="2"/>
       <c r="AF1" s="2"/>
@@ -1505,44 +1520,44 @@
       <c r="AP1" s="3"/>
     </row>
     <row r="2" spans="1:42" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="18"/>
+      <c r="A2" s="38"/>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
-      <c r="K2" s="21"/>
-      <c r="L2" s="21"/>
-      <c r="M2" s="21"/>
-      <c r="N2" s="21"/>
-      <c r="O2" s="21"/>
-      <c r="P2" s="21"/>
-      <c r="Q2" s="21"/>
-      <c r="R2" s="21"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="21"/>
-      <c r="U2" s="21"/>
-      <c r="V2" s="21"/>
-      <c r="W2" s="21"/>
-      <c r="X2" s="21"/>
-      <c r="Y2" s="21"/>
-      <c r="Z2" s="21"/>
-      <c r="AA2" s="21"/>
-      <c r="AB2" s="21"/>
-      <c r="AC2" s="21"/>
-      <c r="AD2" s="21"/>
-      <c r="AE2" s="21"/>
-      <c r="AF2" s="21"/>
-      <c r="AG2" s="21"/>
-      <c r="AH2" s="21"/>
-      <c r="AI2" s="21"/>
-      <c r="AJ2" s="22"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="36"/>
+      <c r="I2" s="36"/>
+      <c r="J2" s="36"/>
+      <c r="K2" s="36"/>
+      <c r="L2" s="36"/>
+      <c r="M2" s="36"/>
+      <c r="N2" s="36"/>
+      <c r="O2" s="36"/>
+      <c r="P2" s="36"/>
+      <c r="Q2" s="36"/>
+      <c r="R2" s="36"/>
+      <c r="S2" s="36"/>
+      <c r="T2" s="36"/>
+      <c r="U2" s="36"/>
+      <c r="V2" s="36"/>
+      <c r="W2" s="36"/>
+      <c r="X2" s="36"/>
+      <c r="Y2" s="36"/>
+      <c r="Z2" s="36"/>
+      <c r="AA2" s="36"/>
+      <c r="AB2" s="36"/>
+      <c r="AC2" s="36"/>
+      <c r="AD2" s="36"/>
+      <c r="AE2" s="36"/>
+      <c r="AF2" s="36"/>
+      <c r="AG2" s="36"/>
+      <c r="AH2" s="36"/>
+      <c r="AI2" s="36"/>
+      <c r="AJ2" s="28"/>
       <c r="AK2" s="3"/>
       <c r="AL2" s="3"/>
       <c r="AM2" s="3"/>
@@ -1551,50 +1566,50 @@
       <c r="AP2" s="3"/>
     </row>
     <row r="3" spans="1:42" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="19"/>
+      <c r="A3" s="39"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="25"/>
-      <c r="J3" s="23" t="s">
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="42"/>
+      <c r="J3" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="25"/>
-      <c r="P3" s="23" t="s">
+      <c r="K3" s="41"/>
+      <c r="L3" s="41"/>
+      <c r="M3" s="41"/>
+      <c r="N3" s="41"/>
+      <c r="O3" s="42"/>
+      <c r="P3" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="Q3" s="24"/>
-      <c r="R3" s="24"/>
-      <c r="S3" s="24"/>
-      <c r="T3" s="24"/>
-      <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
-      <c r="W3" s="24"/>
-      <c r="X3" s="24"/>
-      <c r="Y3" s="24"/>
-      <c r="Z3" s="24"/>
-      <c r="AA3" s="24"/>
-      <c r="AB3" s="24"/>
-      <c r="AC3" s="24"/>
-      <c r="AD3" s="24"/>
-      <c r="AE3" s="24"/>
-      <c r="AF3" s="24"/>
-      <c r="AG3" s="25"/>
-      <c r="AH3" s="23" t="s">
+      <c r="Q3" s="41"/>
+      <c r="R3" s="41"/>
+      <c r="S3" s="41"/>
+      <c r="T3" s="41"/>
+      <c r="U3" s="41"/>
+      <c r="V3" s="41"/>
+      <c r="W3" s="41"/>
+      <c r="X3" s="41"/>
+      <c r="Y3" s="41"/>
+      <c r="Z3" s="41"/>
+      <c r="AA3" s="41"/>
+      <c r="AB3" s="41"/>
+      <c r="AC3" s="41"/>
+      <c r="AD3" s="41"/>
+      <c r="AE3" s="41"/>
+      <c r="AF3" s="41"/>
+      <c r="AG3" s="42"/>
+      <c r="AH3" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="AI3" s="24"/>
-      <c r="AJ3" s="25"/>
+      <c r="AI3" s="41"/>
+      <c r="AJ3" s="42"/>
       <c r="AK3" s="3"/>
       <c r="AL3" s="3"/>
       <c r="AM3" s="3"/>
@@ -1630,8 +1645,8 @@
       <c r="Y4" s="7"/>
       <c r="Z4" s="7"/>
       <c r="AA4" s="7"/>
-      <c r="AB4" s="42"/>
-      <c r="AC4" s="42"/>
+      <c r="AB4" s="18"/>
+      <c r="AC4" s="18"/>
       <c r="AD4" s="7"/>
       <c r="AE4" s="7"/>
       <c r="AF4" s="7"/>
@@ -1652,47 +1667,47 @@
       </c>
       <c r="B5" s="9"/>
       <c r="C5" s="9"/>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27"/>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="28"/>
-      <c r="P5" s="20" t="s">
+      <c r="E5" s="44"/>
+      <c r="F5" s="44"/>
+      <c r="G5" s="44"/>
+      <c r="H5" s="44"/>
+      <c r="I5" s="44"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="44"/>
+      <c r="L5" s="44"/>
+      <c r="M5" s="44"/>
+      <c r="N5" s="44"/>
+      <c r="O5" s="45"/>
+      <c r="P5" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="26" t="s">
+      <c r="Q5" s="36"/>
+      <c r="R5" s="36"/>
+      <c r="S5" s="28"/>
+      <c r="T5" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="U5" s="27"/>
-      <c r="V5" s="27"/>
-      <c r="W5" s="27"/>
-      <c r="X5" s="28"/>
-      <c r="Y5" s="20" t="s">
+      <c r="U5" s="44"/>
+      <c r="V5" s="44"/>
+      <c r="W5" s="44"/>
+      <c r="X5" s="45"/>
+      <c r="Y5" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="Z5" s="22"/>
-      <c r="AA5" s="29"/>
-      <c r="AB5" s="30"/>
-      <c r="AC5" s="30"/>
-      <c r="AD5" s="30"/>
-      <c r="AE5" s="30"/>
-      <c r="AF5" s="30"/>
-      <c r="AG5" s="30"/>
-      <c r="AH5" s="30"/>
-      <c r="AI5" s="30"/>
-      <c r="AJ5" s="31"/>
+      <c r="Z5" s="28"/>
+      <c r="AA5" s="33"/>
+      <c r="AB5" s="34"/>
+      <c r="AC5" s="34"/>
+      <c r="AD5" s="34"/>
+      <c r="AE5" s="34"/>
+      <c r="AF5" s="34"/>
+      <c r="AG5" s="34"/>
+      <c r="AH5" s="34"/>
+      <c r="AI5" s="34"/>
+      <c r="AJ5" s="35"/>
       <c r="AK5" s="10"/>
       <c r="AL5" s="10"/>
       <c r="AM5" s="10"/>
@@ -1728,8 +1743,8 @@
       <c r="Y6" s="7"/>
       <c r="Z6" s="7"/>
       <c r="AA6" s="7"/>
-      <c r="AB6" s="42"/>
-      <c r="AC6" s="42"/>
+      <c r="AB6" s="18"/>
+      <c r="AC6" s="18"/>
       <c r="AD6" s="7"/>
       <c r="AE6" s="7"/>
       <c r="AF6" s="7"/>
@@ -1745,118 +1760,118 @@
       <c r="AP6" s="11"/>
     </row>
     <row r="7" spans="1:42" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="15" t="s">
+      <c r="C7" s="25" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="E7" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="G7" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="35" t="s">
+      <c r="H7" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="35" t="s">
+      <c r="I7" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="35" t="s">
+      <c r="J7" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="K7" s="20" t="s">
+      <c r="K7" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="L7" s="21"/>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21"/>
-      <c r="O7" s="21"/>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="22"/>
-      <c r="T7" s="35" t="s">
+      <c r="L7" s="36"/>
+      <c r="M7" s="36"/>
+      <c r="N7" s="36"/>
+      <c r="O7" s="36"/>
+      <c r="P7" s="36"/>
+      <c r="Q7" s="36"/>
+      <c r="R7" s="36"/>
+      <c r="S7" s="28"/>
+      <c r="T7" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="U7" s="35" t="s">
+      <c r="U7" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="V7" s="35" t="s">
+      <c r="V7" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="W7" s="20" t="s">
+      <c r="W7" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="X7" s="22"/>
-      <c r="Y7" s="35" t="s">
+      <c r="X7" s="28"/>
+      <c r="Y7" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="Z7" s="15" t="s">
+      <c r="Z7" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="AA7" s="15" t="s">
+      <c r="AA7" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="AB7" s="43" t="s">
+      <c r="AB7" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="AC7" s="43" t="s">
+      <c r="AC7" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="AD7" s="20" t="s">
+      <c r="AD7" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="AE7" s="22"/>
-      <c r="AF7" s="35" t="s">
+      <c r="AE7" s="28"/>
+      <c r="AF7" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="AG7" s="35" t="s">
+      <c r="AG7" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="AH7" s="35" t="s">
+      <c r="AH7" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="AI7" s="35" t="s">
+      <c r="AI7" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="AJ7" s="15" t="s">
+      <c r="AJ7" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="AK7" s="37" t="s">
+      <c r="AK7" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="AL7" s="32" t="s">
+      <c r="AL7" s="22" t="s">
         <v>35</v>
       </c>
-      <c r="AM7" s="33"/>
-      <c r="AN7" s="32" t="s">
+      <c r="AM7" s="23"/>
+      <c r="AN7" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="AO7" s="34"/>
-      <c r="AP7" s="33"/>
+      <c r="AO7" s="24"/>
+      <c r="AP7" s="23"/>
     </row>
     <row r="8" spans="1:42" ht="68" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="16"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="36"/>
+      <c r="A8" s="26"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
@@ -1866,45 +1881,45 @@
       <c r="Q8" s="7"/>
       <c r="R8" s="7"/>
       <c r="S8" s="7"/>
-      <c r="T8" s="36"/>
-      <c r="U8" s="36"/>
-      <c r="V8" s="36"/>
-      <c r="W8" s="39" t="s">
+      <c r="T8" s="30"/>
+      <c r="U8" s="30"/>
+      <c r="V8" s="30"/>
+      <c r="W8" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="X8" s="39" t="s">
+      <c r="X8" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="Y8" s="36"/>
-      <c r="Z8" s="16"/>
-      <c r="AA8" s="16"/>
-      <c r="AB8" s="44"/>
-      <c r="AC8" s="44"/>
+      <c r="Y8" s="30"/>
+      <c r="Z8" s="26"/>
+      <c r="AA8" s="26"/>
+      <c r="AB8" s="32"/>
+      <c r="AC8" s="32"/>
       <c r="AD8" s="12" t="s">
         <v>39</v>
       </c>
       <c r="AE8" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="AF8" s="36"/>
-      <c r="AG8" s="36"/>
-      <c r="AH8" s="36"/>
-      <c r="AI8" s="36"/>
-      <c r="AJ8" s="16"/>
-      <c r="AK8" s="38"/>
-      <c r="AL8" s="40" t="s">
+      <c r="AF8" s="30"/>
+      <c r="AG8" s="30"/>
+      <c r="AH8" s="30"/>
+      <c r="AI8" s="30"/>
+      <c r="AJ8" s="26"/>
+      <c r="AK8" s="21"/>
+      <c r="AL8" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="AM8" s="40" t="s">
+      <c r="AM8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AN8" s="40" t="s">
+      <c r="AN8" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="AO8" s="40" t="s">
+      <c r="AO8" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="AP8" s="40" t="s">
+      <c r="AP8" s="16" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1913,6 +1928,30 @@
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="D2:AJ2"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="J3:O3"/>
+    <mergeCell ref="P3:AG3"/>
+    <mergeCell ref="AH3:AJ3"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="D5:O5"/>
+    <mergeCell ref="P5:S5"/>
+    <mergeCell ref="T5:X5"/>
+    <mergeCell ref="Y5:Z5"/>
+    <mergeCell ref="AA5:AJ5"/>
+    <mergeCell ref="AC7:AC8"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="K7:S7"/>
+    <mergeCell ref="T7:T8"/>
+    <mergeCell ref="U7:U8"/>
+    <mergeCell ref="V7:V8"/>
     <mergeCell ref="AK7:AK8"/>
     <mergeCell ref="AL7:AM7"/>
     <mergeCell ref="AN7:AP7"/>
@@ -1929,30 +1968,6 @@
     <mergeCell ref="Z7:Z8"/>
     <mergeCell ref="AA7:AA8"/>
     <mergeCell ref="AB7:AB8"/>
-    <mergeCell ref="AA5:AJ5"/>
-    <mergeCell ref="AC7:AC8"/>
-    <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="K7:S7"/>
-    <mergeCell ref="T7:T8"/>
-    <mergeCell ref="U7:U8"/>
-    <mergeCell ref="V7:V8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="D2:AJ2"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="J3:O3"/>
-    <mergeCell ref="P3:AG3"/>
-    <mergeCell ref="AH3:AJ3"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="F7:F8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="D5:O5"/>
-    <mergeCell ref="P5:S5"/>
-    <mergeCell ref="T5:X5"/>
-    <mergeCell ref="Y5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>